<commit_message>
Guard deprecated latent demand bases; fix doc-code parity
latent_low (38.47) / latent_high (76.93) were derived as 23.08/lambda from
COLLECTED energy (a revenue quantity), not demand. load_scenario now raises
rather than returning them. The only iteration path,
optimize_experiments.py:2698 (run_all_deterministic_scenarios), is legacy
non-LP code with no callers.

Doc-code parity: the demand_level_scenarios docstring attributed the corrected
37.09 value to the superseded NBS Q1 2024 annualised source. Reattributed to
NERC 2024 gross generation. Module docstring carried two contradictory
base-year sections and three copies of the deprecation note; consolidated, with
the 23.08 provenance retained.

data/demand/README.md still presented 23.08 and the lambda derivations as
current; marked SUPERSEDED at the head and retained as provenance. Nothing in
src/ or scripts/ reads the stale demand CSVs.

Baseline objective unchanged at 1.6135585e10.
</commit_message>
<xml_diff>
--- a/data/gas/processed/thermal_generation_2025.xlsx
+++ b/data/gas/processed/thermal_generation_2025.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\MSc\AUST\Thesis\thesis-repo\thesis-code\data\gas\processed\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABAD71C-76B0-43A7-AF04-6A9B6BC555B4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{27EC2458-5580-45E1-A392-D029CE169676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="10980" yWindow="156" windowWidth="11724" windowHeight="12228" xr2:uid="{92C16D02-A4AD-4680-A825-9F62DC52AD19}"/>
+    <workbookView xWindow="10980" yWindow="132" windowWidth="11724" windowHeight="12228" xr2:uid="{92C16D02-A4AD-4680-A825-9F62DC52AD19}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet2" sheetId="2" r:id="rId1"/>
@@ -447,7 +447,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9747CE26-BF7B-4AC2-9CB5-9D5300B2B5D5}">
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G16"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="3" max="3" width="23.21875" bestFit="1" customWidth="1"/>
@@ -564,6 +564,12 @@
         <v>16</v>
       </c>
     </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <f>74.05%*8887.93</f>
+        <v>6581.5121650000001</v>
+      </c>
+    </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="E3" r:id="rId1" xr:uid="{8002BB33-5BA9-4B62-8D62-1E62F56AF786}"/>

</xml_diff>